<commit_message>
Move Beyza Caa Hücre Box 2
</commit_message>
<xml_diff>
--- a/cellstocks/data/admin.xlsx
+++ b/cellstocks/data/admin.xlsx
@@ -37403,17 +37403,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Freezer 2</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Beyza Shelf</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">LiqNitro 1</t>
+          <t xml:space="preserve">Beyza Caa Hücre Box 2</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -37450,7 +37450,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">LiqNitro 2</t>
+          <t xml:space="preserve">LiqNitro 1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -37487,7 +37487,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Beyza Caa Hücre Box 1</t>
+          <t xml:space="preserve">LiqNitro 2</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -37524,7 +37524,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Beyza Caa Sıvı Azot Box 1</t>
+          <t xml:space="preserve">Beyza Caa Hücre Box 1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -37561,7 +37561,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Beyza Caa Hücre Box 2</t>
+          <t xml:space="preserve">Beyza Caa Sıvı Azot Box 1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">

</xml_diff>

<commit_message>
Move Beyza Caa Hücre Box 1
</commit_message>
<xml_diff>
--- a/cellstocks/data/admin.xlsx
+++ b/cellstocks/data/admin.xlsx
@@ -37255,17 +37255,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 2</t>
+          <t xml:space="preserve">Liquid Nitrogen</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Baris Shelf</t>
+          <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">-80 Box1</t>
+          <t xml:space="preserve">Beyza Caa Hücre Box 1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -37302,7 +37302,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">-80 Box2</t>
+          <t xml:space="preserve">-80 Box1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -37339,7 +37339,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">-80 Box3</t>
+          <t xml:space="preserve">-80 Box2</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -37376,7 +37376,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">-80 Box4</t>
+          <t xml:space="preserve">-80 Box3</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -37413,7 +37413,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">-80 Box5</t>
+          <t xml:space="preserve">-80 Box4</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -37450,7 +37450,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">-80 Box6</t>
+          <t xml:space="preserve">-80 Box5</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -37482,12 +37482,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Beyza Shelf</t>
+          <t xml:space="preserve">Baris Shelf</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Beyza Caa Hücre Box 2</t>
+          <t xml:space="preserve">-80 Box6</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -37514,17 +37514,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Freezer 2</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Beyza Shelf</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Beyza Caa Hücre Box 1</t>
+          <t xml:space="preserve">Beyza Caa Hücre Box 2</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">

</xml_diff>

<commit_message>
Move Beyza Caa Sıvı Azot Box 1
</commit_message>
<xml_diff>
--- a/cellstocks/data/admin.xlsx
+++ b/cellstocks/data/admin.xlsx
@@ -37292,17 +37292,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 2</t>
+          <t xml:space="preserve">Liquid Nitrogen</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Baris Shelf</t>
+          <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">-80 Box1</t>
+          <t xml:space="preserve">Beyza Caa Sıvı Azot Box 1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -37339,7 +37339,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">-80 Box2</t>
+          <t xml:space="preserve">-80 Box1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -37376,7 +37376,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">-80 Box3</t>
+          <t xml:space="preserve">-80 Box2</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -37413,7 +37413,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">-80 Box4</t>
+          <t xml:space="preserve">-80 Box3</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -37450,7 +37450,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">-80 Box5</t>
+          <t xml:space="preserve">-80 Box4</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -37487,7 +37487,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">-80 Box6</t>
+          <t xml:space="preserve">-80 Box5</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -37519,12 +37519,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Beyza Shelf</t>
+          <t xml:space="preserve">Baris Shelf</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Beyza Caa Hücre Box 2</t>
+          <t xml:space="preserve">-80 Box6</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -37551,17 +37551,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Freezer 2</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Beyza Shelf</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Beyza Caa Sıvı Azot Box 1</t>
+          <t xml:space="preserve">Beyza Caa Hücre Box 2</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">

</xml_diff>

<commit_message>
Edit a koox rule
</commit_message>
<xml_diff>
--- a/cellstocks/data/admin.xlsx
+++ b/cellstocks/data/admin.xlsx
@@ -201,7 +201,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -283,7 +283,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -365,7 +365,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -447,7 +447,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -529,7 +529,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -611,7 +611,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -775,7 +775,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -857,7 +857,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -939,7 +939,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1021,7 +1021,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1103,7 +1103,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1267,7 +1267,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1349,7 +1349,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1513,7 +1513,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -1595,7 +1595,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -1677,7 +1677,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -1759,7 +1759,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -1841,7 +1841,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -1923,7 +1923,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2005,7 +2005,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -2087,7 +2087,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -2169,7 +2169,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -2251,7 +2251,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -2415,7 +2415,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -2497,7 +2497,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -2579,7 +2579,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -2661,7 +2661,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -2753,7 +2753,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -2845,7 +2845,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -2937,7 +2937,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -3029,7 +3029,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -3111,7 +3111,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -3603,7 +3603,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -4013,7 +4013,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
@@ -4177,7 +4177,7 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
@@ -4259,7 +4259,7 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
@@ -4423,7 +4423,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
@@ -4505,7 +4505,7 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
@@ -4587,7 +4587,7 @@
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
@@ -4669,7 +4669,7 @@
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
@@ -4751,7 +4751,7 @@
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
@@ -4833,7 +4833,7 @@
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
@@ -4915,7 +4915,7 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
@@ -5007,7 +5007,7 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
@@ -5191,7 +5191,7 @@
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
@@ -5283,7 +5283,7 @@
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
@@ -5365,7 +5365,7 @@
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
@@ -5447,7 +5447,7 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
@@ -5529,7 +5529,7 @@
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
@@ -5611,7 +5611,7 @@
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M67" t="inlineStr">
@@ -5693,7 +5693,7 @@
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M68" t="inlineStr">
@@ -5775,7 +5775,7 @@
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M69" t="inlineStr">
@@ -5867,7 +5867,7 @@
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M70" t="inlineStr">
@@ -5949,7 +5949,7 @@
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M71" t="inlineStr">
@@ -6031,7 +6031,7 @@
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M72" t="inlineStr">
@@ -6113,7 +6113,7 @@
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M73" t="inlineStr">
@@ -6523,7 +6523,7 @@
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M78" t="inlineStr">
@@ -6605,7 +6605,7 @@
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M79" t="inlineStr">
@@ -6687,7 +6687,7 @@
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M80" t="inlineStr">
@@ -6769,7 +6769,7 @@
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M81" t="inlineStr">
@@ -6851,7 +6851,7 @@
       </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M82" t="inlineStr">
@@ -6933,7 +6933,7 @@
       </c>
       <c r="L83" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M83" t="inlineStr">
@@ -7015,7 +7015,7 @@
       </c>
       <c r="L84" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M84" t="inlineStr">
@@ -7097,7 +7097,7 @@
       </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M85" t="inlineStr">
@@ -7179,7 +7179,7 @@
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M86" t="inlineStr">
@@ -7343,7 +7343,7 @@
       </c>
       <c r="L88" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M88" t="inlineStr">
@@ -7435,7 +7435,7 @@
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M89" t="inlineStr">
@@ -8173,7 +8173,7 @@
       </c>
       <c r="L98" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M98" t="inlineStr">
@@ -8501,7 +8501,7 @@
       </c>
       <c r="L102" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M102" t="inlineStr">
@@ -8583,7 +8583,7 @@
       </c>
       <c r="L103" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M103" t="inlineStr">
@@ -8665,7 +8665,7 @@
       </c>
       <c r="L104" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M104" t="inlineStr">
@@ -9167,7 +9167,7 @@
       </c>
       <c r="L110" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M110" t="inlineStr">
@@ -9331,7 +9331,7 @@
       </c>
       <c r="L112" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M112" t="inlineStr">
@@ -9413,7 +9413,7 @@
       </c>
       <c r="L113" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M113" t="inlineStr">
@@ -9495,7 +9495,7 @@
       </c>
       <c r="L114" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M114" t="inlineStr">
@@ -9577,7 +9577,7 @@
       </c>
       <c r="L115" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M115" t="inlineStr">
@@ -9659,7 +9659,7 @@
       </c>
       <c r="L116" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M116" t="inlineStr">
@@ -9741,7 +9741,7 @@
       </c>
       <c r="L117" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M117" t="inlineStr">
@@ -9823,7 +9823,7 @@
       </c>
       <c r="L118" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M118" t="inlineStr">
@@ -9905,7 +9905,7 @@
       </c>
       <c r="L119" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M119" t="inlineStr">
@@ -10151,7 +10151,7 @@
       </c>
       <c r="L122" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M122" t="inlineStr">
@@ -10233,7 +10233,7 @@
       </c>
       <c r="L123" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M123" t="inlineStr">
@@ -10315,7 +10315,7 @@
       </c>
       <c r="L124" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M124" t="inlineStr">
@@ -10397,7 +10397,7 @@
       </c>
       <c r="L125" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M125" t="inlineStr">
@@ -10479,7 +10479,7 @@
       </c>
       <c r="L126" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M126" t="inlineStr">
@@ -10561,7 +10561,7 @@
       </c>
       <c r="L127" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M127" t="inlineStr">
@@ -10643,7 +10643,7 @@
       </c>
       <c r="L128" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M128" t="inlineStr">
@@ -10725,7 +10725,7 @@
       </c>
       <c r="L129" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M129" t="inlineStr">
@@ -10807,7 +10807,7 @@
       </c>
       <c r="L130" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M130" t="inlineStr">
@@ -10889,7 +10889,7 @@
       </c>
       <c r="L131" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M131" t="inlineStr">
@@ -10971,7 +10971,7 @@
       </c>
       <c r="L132" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M132" t="inlineStr">
@@ -11053,7 +11053,7 @@
       </c>
       <c r="L133" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M133" t="inlineStr">
@@ -11135,7 +11135,7 @@
       </c>
       <c r="L134" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M134" t="inlineStr">
@@ -11217,7 +11217,7 @@
       </c>
       <c r="L135" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M135" t="inlineStr">
@@ -11299,7 +11299,7 @@
       </c>
       <c r="L136" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M136" t="inlineStr">
@@ -11381,7 +11381,7 @@
       </c>
       <c r="L137" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M137" t="inlineStr">
@@ -11463,7 +11463,7 @@
       </c>
       <c r="L138" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M138" t="inlineStr">
@@ -11545,7 +11545,7 @@
       </c>
       <c r="L139" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M139" t="inlineStr">
@@ -11627,7 +11627,7 @@
       </c>
       <c r="L140" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M140" t="inlineStr">
@@ -11709,7 +11709,7 @@
       </c>
       <c r="L141" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M141" t="inlineStr">
@@ -11791,7 +11791,7 @@
       </c>
       <c r="L142" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M142" t="inlineStr">
@@ -11873,7 +11873,7 @@
       </c>
       <c r="L143" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M143" t="inlineStr">
@@ -11955,7 +11955,7 @@
       </c>
       <c r="L144" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M144" t="inlineStr">
@@ -12037,7 +12037,7 @@
       </c>
       <c r="L145" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M145" t="inlineStr">
@@ -12119,7 +12119,7 @@
       </c>
       <c r="L146" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M146" t="inlineStr">
@@ -12201,7 +12201,7 @@
       </c>
       <c r="L147" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M147" t="inlineStr">
@@ -12283,7 +12283,7 @@
       </c>
       <c r="L148" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M148" t="inlineStr">
@@ -12365,7 +12365,7 @@
       </c>
       <c r="L149" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M149" t="inlineStr">
@@ -12447,7 +12447,7 @@
       </c>
       <c r="L150" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M150" t="inlineStr">
@@ -12529,7 +12529,7 @@
       </c>
       <c r="L151" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M151" t="inlineStr">
@@ -12611,7 +12611,7 @@
       </c>
       <c r="L152" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M152" t="inlineStr">
@@ -13866,7 +13866,7 @@
       </c>
       <c r="L167" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M167" t="inlineStr">
@@ -14112,7 +14112,7 @@
       </c>
       <c r="L170" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M170" t="inlineStr">
@@ -14194,7 +14194,7 @@
       </c>
       <c r="L171" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M171" t="inlineStr">
@@ -14522,7 +14522,7 @@
       </c>
       <c r="L175" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M175" t="inlineStr">
@@ -14604,7 +14604,7 @@
       </c>
       <c r="L176" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M176" t="inlineStr">
@@ -14686,7 +14686,7 @@
       </c>
       <c r="L177" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M177" t="inlineStr">
@@ -14768,7 +14768,7 @@
       </c>
       <c r="L178" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M178" t="inlineStr">
@@ -14932,7 +14932,7 @@
       </c>
       <c r="L180" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M180" t="inlineStr">
@@ -15014,7 +15014,7 @@
       </c>
       <c r="L181" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M181" t="inlineStr">
@@ -15106,7 +15106,7 @@
       </c>
       <c r="L182" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M182" t="inlineStr">
@@ -15188,7 +15188,7 @@
       </c>
       <c r="L183" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M183" t="inlineStr">
@@ -15270,7 +15270,7 @@
       </c>
       <c r="L184" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M184" t="inlineStr">
@@ -15362,7 +15362,7 @@
       </c>
       <c r="L185" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M185" t="inlineStr">
@@ -15454,7 +15454,7 @@
       </c>
       <c r="L186" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M186" t="inlineStr">
@@ -15546,7 +15546,7 @@
       </c>
       <c r="L187" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M187" t="inlineStr">
@@ -15628,7 +15628,7 @@
       </c>
       <c r="L188" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M188" t="inlineStr">
@@ -16120,7 +16120,7 @@
       </c>
       <c r="L194" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M194" t="inlineStr">
@@ -16284,7 +16284,7 @@
       </c>
       <c r="L196" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M196" t="inlineStr">
@@ -16366,7 +16366,7 @@
       </c>
       <c r="L197" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M197" t="inlineStr">
@@ -16448,7 +16448,7 @@
       </c>
       <c r="L198" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M198" t="inlineStr">
@@ -16530,7 +16530,7 @@
       </c>
       <c r="L199" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M199" t="inlineStr">
@@ -16612,7 +16612,7 @@
       </c>
       <c r="L200" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M200" t="inlineStr">
@@ -16694,7 +16694,7 @@
       </c>
       <c r="L201" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M201" t="inlineStr">
@@ -16776,7 +16776,7 @@
       </c>
       <c r="L202" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M202" t="inlineStr">
@@ -16858,7 +16858,7 @@
       </c>
       <c r="L203" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M203" t="inlineStr">
@@ -16940,7 +16940,7 @@
       </c>
       <c r="L204" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M204" t="inlineStr">
@@ -17022,7 +17022,7 @@
       </c>
       <c r="L205" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M205" t="inlineStr">
@@ -17104,7 +17104,7 @@
       </c>
       <c r="L206" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M206" t="inlineStr">
@@ -17186,7 +17186,7 @@
       </c>
       <c r="L207" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M207" t="inlineStr">
@@ -17268,7 +17268,7 @@
       </c>
       <c r="L208" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M208" t="inlineStr">
@@ -17350,7 +17350,7 @@
       </c>
       <c r="L209" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M209" t="inlineStr">
@@ -17432,7 +17432,7 @@
       </c>
       <c r="L210" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M210" t="inlineStr">
@@ -17514,7 +17514,7 @@
       </c>
       <c r="L211" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M211" t="inlineStr">
@@ -17606,7 +17606,7 @@
       </c>
       <c r="L212" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M212" t="inlineStr">
@@ -17688,7 +17688,7 @@
       </c>
       <c r="L213" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M213" t="inlineStr">
@@ -17770,7 +17770,7 @@
       </c>
       <c r="L214" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M214" t="inlineStr">
@@ -17862,7 +17862,7 @@
       </c>
       <c r="L215" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M215" t="inlineStr">
@@ -19266,7 +19266,7 @@
       </c>
       <c r="L232" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M232" t="inlineStr">
@@ -19348,7 +19348,7 @@
       </c>
       <c r="L233" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M233" t="inlineStr">
@@ -19594,7 +19594,7 @@
       </c>
       <c r="L236" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M236" t="inlineStr">
@@ -19917,7 +19917,7 @@
       </c>
       <c r="L240" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M240" t="inlineStr">
@@ -19994,7 +19994,7 @@
       </c>
       <c r="L241" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M241" t="inlineStr">
@@ -20076,7 +20076,7 @@
       </c>
       <c r="L242" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M242" t="inlineStr">
@@ -20158,7 +20158,7 @@
       </c>
       <c r="L243" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M243" t="inlineStr">
@@ -20240,7 +20240,7 @@
       </c>
       <c r="L244" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M244" t="inlineStr">
@@ -20322,7 +20322,7 @@
       </c>
       <c r="L245" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M245" t="inlineStr">
@@ -20399,7 +20399,7 @@
       </c>
       <c r="L246" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M246" t="inlineStr">
@@ -20481,7 +20481,7 @@
       </c>
       <c r="L247" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M247" t="inlineStr">
@@ -20563,7 +20563,7 @@
       </c>
       <c r="L248" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M248" t="inlineStr">
@@ -20645,7 +20645,7 @@
       </c>
       <c r="L249" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M249" t="inlineStr">
@@ -20727,7 +20727,7 @@
       </c>
       <c r="L250" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M250" t="inlineStr">
@@ -20809,7 +20809,7 @@
       </c>
       <c r="L251" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M251" t="inlineStr">
@@ -20891,7 +20891,7 @@
       </c>
       <c r="L252" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M252" t="inlineStr">
@@ -20973,7 +20973,7 @@
       </c>
       <c r="L253" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M253" t="inlineStr">
@@ -21055,7 +21055,7 @@
       </c>
       <c r="L254" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M254" t="inlineStr">
@@ -21137,7 +21137,7 @@
       </c>
       <c r="L255" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M255" t="inlineStr">
@@ -21219,7 +21219,7 @@
       </c>
       <c r="L256" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M256" t="inlineStr">
@@ -21301,7 +21301,7 @@
       </c>
       <c r="L257" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M257" t="inlineStr">
@@ -21383,7 +21383,7 @@
       </c>
       <c r="L258" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M258" t="inlineStr">
@@ -21629,7 +21629,7 @@
       </c>
       <c r="L261" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M261" t="inlineStr">
@@ -21711,7 +21711,7 @@
       </c>
       <c r="L262" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M262" t="inlineStr">
@@ -21793,7 +21793,7 @@
       </c>
       <c r="L263" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M263" t="inlineStr">
@@ -21875,7 +21875,7 @@
       </c>
       <c r="L264" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M264" t="inlineStr">
@@ -21957,7 +21957,7 @@
       </c>
       <c r="L265" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M265" t="inlineStr">
@@ -22039,7 +22039,7 @@
       </c>
       <c r="L266" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M266" t="inlineStr">
@@ -22116,7 +22116,7 @@
       </c>
       <c r="L267" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M267" t="inlineStr">
@@ -22193,7 +22193,7 @@
       </c>
       <c r="L268" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M268" t="inlineStr">
@@ -22275,7 +22275,7 @@
       </c>
       <c r="L269" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M269" t="inlineStr">
@@ -22357,7 +22357,7 @@
       </c>
       <c r="L270" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M270" t="inlineStr">
@@ -22439,7 +22439,7 @@
       </c>
       <c r="L271" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M271" t="inlineStr">
@@ -22521,7 +22521,7 @@
       </c>
       <c r="L272" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M272" t="inlineStr">
@@ -22603,7 +22603,7 @@
       </c>
       <c r="L273" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M273" t="inlineStr">
@@ -22685,7 +22685,7 @@
       </c>
       <c r="L274" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M274" t="inlineStr">
@@ -22767,7 +22767,7 @@
       </c>
       <c r="L275" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M275" t="inlineStr">
@@ -22849,7 +22849,7 @@
       </c>
       <c r="L276" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M276" t="inlineStr">
@@ -22931,7 +22931,7 @@
       </c>
       <c r="L277" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M277" t="inlineStr">
@@ -23013,7 +23013,7 @@
       </c>
       <c r="L278" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M278" t="inlineStr">
@@ -23095,7 +23095,7 @@
       </c>
       <c r="L279" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M279" t="inlineStr">
@@ -23177,7 +23177,7 @@
       </c>
       <c r="L280" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M280" t="inlineStr">
@@ -23259,7 +23259,7 @@
       </c>
       <c r="L281" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M281" t="inlineStr">
@@ -23341,7 +23341,7 @@
       </c>
       <c r="L282" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M282" t="inlineStr">
@@ -23423,7 +23423,7 @@
       </c>
       <c r="L283" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M283" t="inlineStr">
@@ -23505,7 +23505,7 @@
       </c>
       <c r="L284" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M284" t="inlineStr">
@@ -24320,7 +24320,7 @@
       </c>
       <c r="L294" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M294" t="inlineStr">
@@ -24402,7 +24402,7 @@
       </c>
       <c r="L295" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M295" t="inlineStr">
@@ -24484,7 +24484,7 @@
       </c>
       <c r="L296" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M296" t="inlineStr">
@@ -24648,7 +24648,7 @@
       </c>
       <c r="L298" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M298" t="inlineStr">
@@ -25058,7 +25058,7 @@
       </c>
       <c r="L303" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M303" t="inlineStr">
@@ -25140,7 +25140,7 @@
       </c>
       <c r="L304" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M304" t="inlineStr">
@@ -25222,7 +25222,7 @@
       </c>
       <c r="L305" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M305" t="inlineStr">
@@ -25304,7 +25304,7 @@
       </c>
       <c r="L306" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M306" t="inlineStr">
@@ -25386,7 +25386,7 @@
       </c>
       <c r="L307" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M307" t="inlineStr">
@@ -25468,7 +25468,7 @@
       </c>
       <c r="L308" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M308" t="inlineStr">
@@ -25550,7 +25550,7 @@
       </c>
       <c r="L309" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M309" t="inlineStr">
@@ -25632,7 +25632,7 @@
       </c>
       <c r="L310" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M310" t="inlineStr">
@@ -25714,7 +25714,7 @@
       </c>
       <c r="L311" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M311" t="inlineStr">
@@ -26698,7 +26698,7 @@
       </c>
       <c r="L323" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M323" t="inlineStr">
@@ -26780,7 +26780,7 @@
       </c>
       <c r="L324" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M324" t="inlineStr">
@@ -27190,7 +27190,7 @@
       </c>
       <c r="L329" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M329" t="inlineStr">
@@ -27272,7 +27272,7 @@
       </c>
       <c r="L330" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M330" t="inlineStr">
@@ -27364,7 +27364,7 @@
       </c>
       <c r="L331" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M331" t="inlineStr">
@@ -27456,7 +27456,7 @@
       </c>
       <c r="L332" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M332" t="inlineStr">
@@ -27538,7 +27538,7 @@
       </c>
       <c r="L333" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M333" t="inlineStr">
@@ -27620,7 +27620,7 @@
       </c>
       <c r="L334" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M334" t="inlineStr">
@@ -27702,7 +27702,7 @@
       </c>
       <c r="L335" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M335" t="inlineStr">
@@ -27784,7 +27784,7 @@
       </c>
       <c r="L336" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M336" t="inlineStr">
@@ -27861,7 +27861,7 @@
       </c>
       <c r="L337" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M337" t="inlineStr">
@@ -27943,7 +27943,7 @@
       </c>
       <c r="L338" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M338" t="inlineStr">
@@ -28271,7 +28271,7 @@
       </c>
       <c r="L342" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M342" t="inlineStr">
@@ -28353,7 +28353,7 @@
       </c>
       <c r="L343" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M343" t="inlineStr">
@@ -28435,7 +28435,7 @@
       </c>
       <c r="L344" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M344" t="inlineStr">
@@ -28763,7 +28763,7 @@
       </c>
       <c r="L348" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M348" t="inlineStr">
@@ -28845,7 +28845,7 @@
       </c>
       <c r="L349" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M349" t="inlineStr">
@@ -28927,7 +28927,7 @@
       </c>
       <c r="L350" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M350" t="inlineStr">
@@ -29009,7 +29009,7 @@
       </c>
       <c r="L351" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M351" t="inlineStr">
@@ -29091,7 +29091,7 @@
       </c>
       <c r="L352" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M352" t="inlineStr">
@@ -29173,7 +29173,7 @@
       </c>
       <c r="L353" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M353" t="inlineStr">
@@ -29255,7 +29255,7 @@
       </c>
       <c r="L354" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M354" t="inlineStr">
@@ -29337,7 +29337,7 @@
       </c>
       <c r="L355" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M355" t="inlineStr">
@@ -29419,7 +29419,7 @@
       </c>
       <c r="L356" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M356" t="inlineStr">
@@ -29481,7 +29481,7 @@
       </c>
       <c r="L357" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M357" t="inlineStr">
@@ -29543,7 +29543,7 @@
       </c>
       <c r="L358" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M358" t="inlineStr">
@@ -29791,7 +29791,7 @@
       </c>
       <c r="L362" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M362" t="inlineStr">
@@ -30039,7 +30039,7 @@
       </c>
       <c r="L366" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M366" t="inlineStr">
@@ -30143,7 +30143,7 @@
       </c>
       <c r="L368" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M368" t="inlineStr">
@@ -30195,7 +30195,7 @@
       </c>
       <c r="L369" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M369" t="inlineStr">
@@ -30247,7 +30247,7 @@
       </c>
       <c r="L370" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M370" t="inlineStr">
@@ -30299,7 +30299,7 @@
       </c>
       <c r="L371" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M371" t="inlineStr">
@@ -30351,7 +30351,7 @@
       </c>
       <c r="L372" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M372" t="inlineStr">
@@ -30403,7 +30403,7 @@
       </c>
       <c r="L373" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M373" t="inlineStr">
@@ -30455,7 +30455,7 @@
       </c>
       <c r="L374" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M374" t="inlineStr">
@@ -30512,7 +30512,7 @@
       </c>
       <c r="L375" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M375" t="inlineStr">

</xml_diff>

<commit_message>
Edit a caspex rule
</commit_message>
<xml_diff>
--- a/cellstocks/data/admin.xlsx
+++ b/cellstocks/data/admin.xlsx
@@ -539,7 +539,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -621,7 +621,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -703,7 +703,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -785,7 +785,7 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -1605,7 +1605,7 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
@@ -1687,7 +1687,7 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
@@ -1769,7 +1769,7 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
@@ -1851,7 +1851,7 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
@@ -2015,7 +2015,7 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
@@ -2097,7 +2097,7 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
@@ -2179,7 +2179,7 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
@@ -2261,7 +2261,7 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
@@ -2343,7 +2343,7 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
@@ -2425,7 +2425,7 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
@@ -2507,7 +2507,7 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
@@ -2589,7 +2589,7 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
@@ -2671,7 +2671,7 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
@@ -2763,7 +2763,7 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
@@ -2855,7 +2855,7 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
@@ -3203,7 +3203,7 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
@@ -3285,7 +3285,7 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
@@ -3367,7 +3367,7 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O40" t="inlineStr">
@@ -3449,7 +3449,7 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O41" t="inlineStr">
@@ -3531,7 +3531,7 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
@@ -3613,7 +3613,7 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
@@ -3695,7 +3695,7 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O44" t="inlineStr">
@@ -3777,7 +3777,7 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
@@ -3859,7 +3859,7 @@
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O46" t="inlineStr">
@@ -3941,7 +3941,7 @@
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O47" t="inlineStr">
@@ -4023,7 +4023,7 @@
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O48" t="inlineStr">
@@ -4105,7 +4105,7 @@
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
@@ -4187,7 +4187,7 @@
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
@@ -4269,7 +4269,7 @@
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O51" t="inlineStr">
@@ -4351,7 +4351,7 @@
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O52" t="inlineStr">
@@ -4433,7 +4433,7 @@
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O53" t="inlineStr">
@@ -4679,7 +4679,7 @@
       </c>
       <c r="N56" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O56" t="inlineStr">
@@ -4761,7 +4761,7 @@
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O57" t="inlineStr">
@@ -5293,7 +5293,7 @@
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O63" t="inlineStr">
@@ -5877,7 +5877,7 @@
       </c>
       <c r="N70" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O70" t="inlineStr">
@@ -5959,7 +5959,7 @@
       </c>
       <c r="N71" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O71" t="inlineStr">
@@ -6041,7 +6041,7 @@
       </c>
       <c r="N72" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O72" t="inlineStr">
@@ -6123,7 +6123,7 @@
       </c>
       <c r="N73" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O73" t="inlineStr">
@@ -6205,7 +6205,7 @@
       </c>
       <c r="N74" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O74" t="inlineStr">
@@ -6287,7 +6287,7 @@
       </c>
       <c r="N75" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O75" t="inlineStr">
@@ -6369,7 +6369,7 @@
       </c>
       <c r="N76" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O76" t="inlineStr">
@@ -6451,7 +6451,7 @@
       </c>
       <c r="N77" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O77" t="inlineStr">
@@ -6615,7 +6615,7 @@
       </c>
       <c r="N79" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O79" t="inlineStr">
@@ -6697,7 +6697,7 @@
       </c>
       <c r="N80" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O80" t="inlineStr">
@@ -6779,7 +6779,7 @@
       </c>
       <c r="N81" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O81" t="inlineStr">
@@ -6861,7 +6861,7 @@
       </c>
       <c r="N82" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O82" t="inlineStr">
@@ -6943,7 +6943,7 @@
       </c>
       <c r="N83" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O83" t="inlineStr">
@@ -7025,7 +7025,7 @@
       </c>
       <c r="N84" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O84" t="inlineStr">
@@ -7107,7 +7107,7 @@
       </c>
       <c r="N85" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O85" t="inlineStr">
@@ -7189,7 +7189,7 @@
       </c>
       <c r="N86" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O86" t="inlineStr">
@@ -7271,7 +7271,7 @@
       </c>
       <c r="N87" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O87" t="inlineStr">
@@ -7353,7 +7353,7 @@
       </c>
       <c r="N88" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O88" t="inlineStr">
@@ -7445,7 +7445,7 @@
       </c>
       <c r="N89" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O89" t="inlineStr">
@@ -7527,7 +7527,7 @@
       </c>
       <c r="N90" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O90" t="inlineStr">
@@ -7609,7 +7609,7 @@
       </c>
       <c r="N91" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O91" t="inlineStr">
@@ -7691,7 +7691,7 @@
       </c>
       <c r="N92" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O92" t="inlineStr">
@@ -7773,7 +7773,7 @@
       </c>
       <c r="N93" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O93" t="inlineStr">
@@ -7855,7 +7855,7 @@
       </c>
       <c r="N94" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O94" t="inlineStr">
@@ -7937,7 +7937,7 @@
       </c>
       <c r="N95" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O95" t="inlineStr">
@@ -8019,7 +8019,7 @@
       </c>
       <c r="N96" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O96" t="inlineStr">
@@ -8101,7 +8101,7 @@
       </c>
       <c r="N97" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O97" t="inlineStr">
@@ -8265,7 +8265,7 @@
       </c>
       <c r="N99" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O99" t="inlineStr">
@@ -8347,7 +8347,7 @@
       </c>
       <c r="N100" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O100" t="inlineStr">
@@ -8429,7 +8429,7 @@
       </c>
       <c r="N101" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O101" t="inlineStr">
@@ -8511,7 +8511,7 @@
       </c>
       <c r="N102" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O102" t="inlineStr">
@@ -8593,7 +8593,7 @@
       </c>
       <c r="N103" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O103" t="inlineStr">
@@ -8675,7 +8675,7 @@
       </c>
       <c r="N104" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O104" t="inlineStr">
@@ -8767,7 +8767,7 @@
       </c>
       <c r="N105" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O105" t="inlineStr">
@@ -8849,7 +8849,7 @@
       </c>
       <c r="N106" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O106" t="inlineStr">
@@ -8931,7 +8931,7 @@
       </c>
       <c r="N107" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O107" t="inlineStr">
@@ -9013,7 +9013,7 @@
       </c>
       <c r="N108" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O108" t="inlineStr">
@@ -9095,7 +9095,7 @@
       </c>
       <c r="N109" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O109" t="inlineStr">
@@ -9177,7 +9177,7 @@
       </c>
       <c r="N110" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O110" t="inlineStr">
@@ -9259,7 +9259,7 @@
       </c>
       <c r="N111" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O111" t="inlineStr">
@@ -9505,7 +9505,7 @@
       </c>
       <c r="N114" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O114" t="inlineStr">
@@ -9587,7 +9587,7 @@
       </c>
       <c r="N115" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O115" t="inlineStr">
@@ -9669,7 +9669,7 @@
       </c>
       <c r="N116" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O116" t="inlineStr">
@@ -9751,7 +9751,7 @@
       </c>
       <c r="N117" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O117" t="inlineStr">
@@ -9915,7 +9915,7 @@
       </c>
       <c r="N119" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O119" t="inlineStr">
@@ -9997,7 +9997,7 @@
       </c>
       <c r="N120" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O120" t="inlineStr">
@@ -10079,7 +10079,7 @@
       </c>
       <c r="N121" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O121" t="inlineStr">
@@ -10161,7 +10161,7 @@
       </c>
       <c r="N122" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O122" t="inlineStr">
@@ -10243,7 +10243,7 @@
       </c>
       <c r="N123" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O123" t="inlineStr">
@@ -10489,7 +10489,7 @@
       </c>
       <c r="N126" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O126" t="inlineStr">
@@ -10571,7 +10571,7 @@
       </c>
       <c r="N127" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O127" t="inlineStr">
@@ -10653,7 +10653,7 @@
       </c>
       <c r="N128" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O128" t="inlineStr">
@@ -10735,7 +10735,7 @@
       </c>
       <c r="N129" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O129" t="inlineStr">
@@ -10817,7 +10817,7 @@
       </c>
       <c r="N130" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O130" t="inlineStr">
@@ -10899,7 +10899,7 @@
       </c>
       <c r="N131" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O131" t="inlineStr">
@@ -10981,7 +10981,7 @@
       </c>
       <c r="N132" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O132" t="inlineStr">
@@ -11063,7 +11063,7 @@
       </c>
       <c r="N133" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O133" t="inlineStr">
@@ -11145,7 +11145,7 @@
       </c>
       <c r="N134" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O134" t="inlineStr">
@@ -11227,7 +11227,7 @@
       </c>
       <c r="N135" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O135" t="inlineStr">
@@ -11309,7 +11309,7 @@
       </c>
       <c r="N136" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O136" t="inlineStr">
@@ -11391,7 +11391,7 @@
       </c>
       <c r="N137" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O137" t="inlineStr">
@@ -11473,7 +11473,7 @@
       </c>
       <c r="N138" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O138" t="inlineStr">
@@ -11555,7 +11555,7 @@
       </c>
       <c r="N139" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O139" t="inlineStr">
@@ -11965,7 +11965,7 @@
       </c>
       <c r="N144" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O144" t="inlineStr">
@@ -12293,7 +12293,7 @@
       </c>
       <c r="N148" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O148" t="inlineStr">
@@ -12375,7 +12375,7 @@
       </c>
       <c r="N149" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O149" t="inlineStr">
@@ -12703,7 +12703,7 @@
       </c>
       <c r="N153" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O153" t="inlineStr">
@@ -12790,7 +12790,7 @@
       </c>
       <c r="N154" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O154" t="inlineStr">
@@ -12877,7 +12877,7 @@
       </c>
       <c r="N155" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O155" t="inlineStr">
@@ -12964,7 +12964,7 @@
       </c>
       <c r="N156" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O156" t="inlineStr">
@@ -13046,7 +13046,7 @@
       </c>
       <c r="N157" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O157" t="inlineStr">
@@ -13128,7 +13128,7 @@
       </c>
       <c r="N158" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O158" t="inlineStr">
@@ -13210,7 +13210,7 @@
       </c>
       <c r="N159" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O159" t="inlineStr">
@@ -13292,7 +13292,7 @@
       </c>
       <c r="N160" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O160" t="inlineStr">
@@ -13374,7 +13374,7 @@
       </c>
       <c r="N161" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O161" t="inlineStr">
@@ -13466,7 +13466,7 @@
       </c>
       <c r="N162" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O162" t="inlineStr">
@@ -13548,7 +13548,7 @@
       </c>
       <c r="N163" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O163" t="inlineStr">
@@ -13630,7 +13630,7 @@
       </c>
       <c r="N164" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O164" t="inlineStr">
@@ -13712,7 +13712,7 @@
       </c>
       <c r="N165" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O165" t="inlineStr">
@@ -13794,7 +13794,7 @@
       </c>
       <c r="N166" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O166" t="inlineStr">
@@ -13876,7 +13876,7 @@
       </c>
       <c r="N167" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O167" t="inlineStr">
@@ -13958,7 +13958,7 @@
       </c>
       <c r="N168" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O168" t="inlineStr">
@@ -14040,7 +14040,7 @@
       </c>
       <c r="N169" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O169" t="inlineStr">
@@ -14122,7 +14122,7 @@
       </c>
       <c r="N170" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O170" t="inlineStr">
@@ -14204,7 +14204,7 @@
       </c>
       <c r="N171" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O171" t="inlineStr">
@@ -14286,7 +14286,7 @@
       </c>
       <c r="N172" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O172" t="inlineStr">
@@ -14368,7 +14368,7 @@
       </c>
       <c r="N173" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O173" t="inlineStr">
@@ -14450,7 +14450,7 @@
       </c>
       <c r="N174" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O174" t="inlineStr">
@@ -14532,7 +14532,7 @@
       </c>
       <c r="N175" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O175" t="inlineStr">
@@ -14614,7 +14614,7 @@
       </c>
       <c r="N176" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O176" t="inlineStr">
@@ -14696,7 +14696,7 @@
       </c>
       <c r="N177" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O177" t="inlineStr">
@@ -14778,7 +14778,7 @@
       </c>
       <c r="N178" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O178" t="inlineStr">
@@ -14860,7 +14860,7 @@
       </c>
       <c r="N179" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O179" t="inlineStr">
@@ -14942,7 +14942,7 @@
       </c>
       <c r="N180" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O180" t="inlineStr">
@@ -15024,7 +15024,7 @@
       </c>
       <c r="N181" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O181" t="inlineStr">
@@ -15198,7 +15198,7 @@
       </c>
       <c r="N183" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O183" t="inlineStr">
@@ -15280,7 +15280,7 @@
       </c>
       <c r="N184" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O184" t="inlineStr">
@@ -15372,7 +15372,7 @@
       </c>
       <c r="N185" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O185" t="inlineStr">
@@ -15464,7 +15464,7 @@
       </c>
       <c r="N186" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O186" t="inlineStr">
@@ -15556,7 +15556,7 @@
       </c>
       <c r="N187" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O187" t="inlineStr">
@@ -15720,7 +15720,7 @@
       </c>
       <c r="N189" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O189" t="inlineStr">
@@ -15802,7 +15802,7 @@
       </c>
       <c r="N190" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O190" t="inlineStr">
@@ -15884,7 +15884,7 @@
       </c>
       <c r="N191" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O191" t="inlineStr">
@@ -15966,7 +15966,7 @@
       </c>
       <c r="N192" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O192" t="inlineStr">
@@ -16048,7 +16048,7 @@
       </c>
       <c r="N193" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O193" t="inlineStr">
@@ -16130,7 +16130,7 @@
       </c>
       <c r="N194" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O194" t="inlineStr">
@@ -16212,7 +16212,7 @@
       </c>
       <c r="N195" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O195" t="inlineStr">
@@ -16458,7 +16458,7 @@
       </c>
       <c r="N198" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O198" t="inlineStr">
@@ -16540,7 +16540,7 @@
       </c>
       <c r="N199" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O199" t="inlineStr">
@@ -16622,7 +16622,7 @@
       </c>
       <c r="N200" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O200" t="inlineStr">
@@ -16704,7 +16704,7 @@
       </c>
       <c r="N201" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O201" t="inlineStr">
@@ -16786,7 +16786,7 @@
       </c>
       <c r="N202" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O202" t="inlineStr">
@@ -16868,7 +16868,7 @@
       </c>
       <c r="N203" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O203" t="inlineStr">
@@ -17114,7 +17114,7 @@
       </c>
       <c r="N206" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O206" t="inlineStr">
@@ -17278,7 +17278,7 @@
       </c>
       <c r="N208" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O208" t="inlineStr">
@@ -17360,7 +17360,7 @@
       </c>
       <c r="N209" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O209" t="inlineStr">
@@ -17442,7 +17442,7 @@
       </c>
       <c r="N210" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O210" t="inlineStr">
@@ -17524,7 +17524,7 @@
       </c>
       <c r="N211" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O211" t="inlineStr">
@@ -17616,7 +17616,7 @@
       </c>
       <c r="N212" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O212" t="inlineStr">
@@ -17698,7 +17698,7 @@
       </c>
       <c r="N213" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O213" t="inlineStr">
@@ -17964,7 +17964,7 @@
       </c>
       <c r="N216" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O216" t="inlineStr">
@@ -18046,7 +18046,7 @@
       </c>
       <c r="N217" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O217" t="inlineStr">
@@ -18128,7 +18128,7 @@
       </c>
       <c r="N218" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O218" t="inlineStr">
@@ -18210,7 +18210,7 @@
       </c>
       <c r="N219" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O219" t="inlineStr">
@@ -18292,7 +18292,7 @@
       </c>
       <c r="N220" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O220" t="inlineStr">
@@ -18374,7 +18374,7 @@
       </c>
       <c r="N221" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O221" t="inlineStr">
@@ -18456,7 +18456,7 @@
       </c>
       <c r="N222" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O222" t="inlineStr">
@@ -18538,7 +18538,7 @@
       </c>
       <c r="N223" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O223" t="inlineStr">
@@ -18620,7 +18620,7 @@
       </c>
       <c r="N224" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O224" t="inlineStr">
@@ -18702,7 +18702,7 @@
       </c>
       <c r="N225" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O225" t="inlineStr">
@@ -18784,7 +18784,7 @@
       </c>
       <c r="N226" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O226" t="inlineStr">
@@ -18866,7 +18866,7 @@
       </c>
       <c r="N227" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O227" t="inlineStr">
@@ -18948,7 +18948,7 @@
       </c>
       <c r="N228" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O228" t="inlineStr">
@@ -19030,7 +19030,7 @@
       </c>
       <c r="N229" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O229" t="inlineStr">
@@ -19112,7 +19112,7 @@
       </c>
       <c r="N230" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O230" t="inlineStr">
@@ -19194,7 +19194,7 @@
       </c>
       <c r="N231" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O231" t="inlineStr">
@@ -19276,7 +19276,7 @@
       </c>
       <c r="N232" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O232" t="inlineStr">
@@ -19358,7 +19358,7 @@
       </c>
       <c r="N233" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O233" t="inlineStr">
@@ -19440,7 +19440,7 @@
       </c>
       <c r="N234" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O234" t="inlineStr">
@@ -19522,7 +19522,7 @@
       </c>
       <c r="N235" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O235" t="inlineStr">
@@ -19604,7 +19604,7 @@
       </c>
       <c r="N236" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O236" t="inlineStr">
@@ -19686,7 +19686,7 @@
       </c>
       <c r="N237" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O237" t="inlineStr">
@@ -19768,7 +19768,7 @@
       </c>
       <c r="N238" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O238" t="inlineStr">
@@ -19850,7 +19850,7 @@
       </c>
       <c r="N239" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O239" t="inlineStr">
@@ -19927,7 +19927,7 @@
       </c>
       <c r="N240" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O240" t="inlineStr">
@@ -20004,7 +20004,7 @@
       </c>
       <c r="N241" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O241" t="inlineStr">
@@ -20086,7 +20086,7 @@
       </c>
       <c r="N242" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O242" t="inlineStr">
@@ -20168,7 +20168,7 @@
       </c>
       <c r="N243" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O243" t="inlineStr">
@@ -20250,7 +20250,7 @@
       </c>
       <c r="N244" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O244" t="inlineStr">
@@ -20332,7 +20332,7 @@
       </c>
       <c r="N245" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O245" t="inlineStr">
@@ -20409,7 +20409,7 @@
       </c>
       <c r="N246" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O246" t="inlineStr">
@@ -20491,7 +20491,7 @@
       </c>
       <c r="N247" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O247" t="inlineStr">
@@ -20573,7 +20573,7 @@
       </c>
       <c r="N248" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O248" t="inlineStr">
@@ -20655,7 +20655,7 @@
       </c>
       <c r="N249" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O249" t="inlineStr">
@@ -20737,7 +20737,7 @@
       </c>
       <c r="N250" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O250" t="inlineStr">
@@ -20819,7 +20819,7 @@
       </c>
       <c r="N251" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O251" t="inlineStr">
@@ -20901,7 +20901,7 @@
       </c>
       <c r="N252" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O252" t="inlineStr">
@@ -21065,7 +21065,7 @@
       </c>
       <c r="N254" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O254" t="inlineStr">
@@ -21147,7 +21147,7 @@
       </c>
       <c r="N255" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O255" t="inlineStr">
@@ -21311,7 +21311,7 @@
       </c>
       <c r="N257" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O257" t="inlineStr">
@@ -21393,7 +21393,7 @@
       </c>
       <c r="N258" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O258" t="inlineStr">
@@ -21475,7 +21475,7 @@
       </c>
       <c r="N259" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O259" t="inlineStr">
@@ -21557,7 +21557,7 @@
       </c>
       <c r="N260" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O260" t="inlineStr">
@@ -22126,7 +22126,7 @@
       </c>
       <c r="N267" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O267" t="inlineStr">
@@ -22203,7 +22203,7 @@
       </c>
       <c r="N268" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O268" t="inlineStr">
@@ -23597,7 +23597,7 @@
       </c>
       <c r="N285" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O285" t="inlineStr">
@@ -23679,7 +23679,7 @@
       </c>
       <c r="N286" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O286" t="inlineStr">
@@ -23761,7 +23761,7 @@
       </c>
       <c r="N287" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O287" t="inlineStr">
@@ -23843,7 +23843,7 @@
       </c>
       <c r="N288" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O288" t="inlineStr">
@@ -23925,7 +23925,7 @@
       </c>
       <c r="N289" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O289" t="inlineStr">
@@ -24007,7 +24007,7 @@
       </c>
       <c r="N290" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O290" t="inlineStr">
@@ -24089,7 +24089,7 @@
       </c>
       <c r="N291" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O291" t="inlineStr">
@@ -24171,7 +24171,7 @@
       </c>
       <c r="N292" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O292" t="inlineStr">
@@ -24253,7 +24253,7 @@
       </c>
       <c r="N293" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O293" t="inlineStr">
@@ -24330,7 +24330,7 @@
       </c>
       <c r="N294" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O294" t="inlineStr">
@@ -24412,7 +24412,7 @@
       </c>
       <c r="N295" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O295" t="inlineStr">
@@ -24494,7 +24494,7 @@
       </c>
       <c r="N296" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O296" t="inlineStr">
@@ -24576,7 +24576,7 @@
       </c>
       <c r="N297" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O297" t="inlineStr">
@@ -24658,7 +24658,7 @@
       </c>
       <c r="N298" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O298" t="inlineStr">
@@ -24740,7 +24740,7 @@
       </c>
       <c r="N299" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O299" t="inlineStr">
@@ -24822,7 +24822,7 @@
       </c>
       <c r="N300" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O300" t="inlineStr">
@@ -24904,7 +24904,7 @@
       </c>
       <c r="N301" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O301" t="inlineStr">
@@ -24986,7 +24986,7 @@
       </c>
       <c r="N302" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O302" t="inlineStr">
@@ -25314,7 +25314,7 @@
       </c>
       <c r="N306" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O306" t="inlineStr">
@@ -25396,7 +25396,7 @@
       </c>
       <c r="N307" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O307" t="inlineStr">
@@ -25806,7 +25806,7 @@
       </c>
       <c r="N312" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O312" t="inlineStr">
@@ -25888,7 +25888,7 @@
       </c>
       <c r="N313" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O313" t="inlineStr">
@@ -25970,7 +25970,7 @@
       </c>
       <c r="N314" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O314" t="inlineStr">
@@ -26052,7 +26052,7 @@
       </c>
       <c r="N315" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O315" t="inlineStr">
@@ -26134,7 +26134,7 @@
       </c>
       <c r="N316" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O316" t="inlineStr">
@@ -26216,7 +26216,7 @@
       </c>
       <c r="N317" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O317" t="inlineStr">
@@ -26298,7 +26298,7 @@
       </c>
       <c r="N318" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O318" t="inlineStr">
@@ -26380,7 +26380,7 @@
       </c>
       <c r="N319" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O319" t="inlineStr">
@@ -26462,7 +26462,7 @@
       </c>
       <c r="N320" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O320" t="inlineStr">
@@ -26544,7 +26544,7 @@
       </c>
       <c r="N321" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O321" t="inlineStr">
@@ -26626,7 +26626,7 @@
       </c>
       <c r="N322" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O322" t="inlineStr">
@@ -26708,7 +26708,7 @@
       </c>
       <c r="N323" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O323" t="inlineStr">
@@ -26790,7 +26790,7 @@
       </c>
       <c r="N324" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O324" t="inlineStr">
@@ -26872,7 +26872,7 @@
       </c>
       <c r="N325" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O325" t="inlineStr">
@@ -26954,7 +26954,7 @@
       </c>
       <c r="N326" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O326" t="inlineStr">
@@ -27036,7 +27036,7 @@
       </c>
       <c r="N327" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O327" t="inlineStr">
@@ -27118,7 +27118,7 @@
       </c>
       <c r="N328" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O328" t="inlineStr">
@@ -27200,7 +27200,7 @@
       </c>
       <c r="N329" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O329" t="inlineStr">
@@ -27630,7 +27630,7 @@
       </c>
       <c r="N334" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O334" t="inlineStr">
@@ -27712,7 +27712,7 @@
       </c>
       <c r="N335" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O335" t="inlineStr">
@@ -27794,7 +27794,7 @@
       </c>
       <c r="N336" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O336" t="inlineStr">
@@ -28035,7 +28035,7 @@
       </c>
       <c r="N339" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O339" t="inlineStr">
@@ -28117,7 +28117,7 @@
       </c>
       <c r="N340" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O340" t="inlineStr">
@@ -28199,7 +28199,7 @@
       </c>
       <c r="N341" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O341" t="inlineStr">
@@ -28281,7 +28281,7 @@
       </c>
       <c r="N342" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O342" t="inlineStr">
@@ -28363,7 +28363,7 @@
       </c>
       <c r="N343" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O343" t="inlineStr">
@@ -28527,7 +28527,7 @@
       </c>
       <c r="N345" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O345" t="inlineStr">
@@ -28609,7 +28609,7 @@
       </c>
       <c r="N346" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O346" t="inlineStr">
@@ -28691,7 +28691,7 @@
       </c>
       <c r="N347" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O347" t="inlineStr">
@@ -29265,7 +29265,7 @@
       </c>
       <c r="N354" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O354" t="inlineStr">
@@ -29347,7 +29347,7 @@
       </c>
       <c r="N355" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O355" t="inlineStr">
@@ -29491,7 +29491,7 @@
       </c>
       <c r="N357" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O357" t="inlineStr">
@@ -29553,7 +29553,7 @@
       </c>
       <c r="N358" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O358" t="inlineStr">
@@ -29615,7 +29615,7 @@
       </c>
       <c r="N359" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O359" t="inlineStr">
@@ -29677,7 +29677,7 @@
       </c>
       <c r="N360" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O360" t="inlineStr">
@@ -29739,7 +29739,7 @@
       </c>
       <c r="N361" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O361" t="inlineStr">
@@ -29801,7 +29801,7 @@
       </c>
       <c r="N362" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O362" t="inlineStr">
@@ -29863,7 +29863,7 @@
       </c>
       <c r="N363" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O363" t="inlineStr">
@@ -29925,7 +29925,7 @@
       </c>
       <c r="N364" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O364" t="inlineStr">
@@ -29987,7 +29987,7 @@
       </c>
       <c r="N365" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O365" t="inlineStr">
@@ -30101,7 +30101,7 @@
       </c>
       <c r="N367" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O367" t="inlineStr">
@@ -30153,7 +30153,7 @@
       </c>
       <c r="N368" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O368" t="inlineStr">
@@ -30205,7 +30205,7 @@
       </c>
       <c r="N369" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O369" t="inlineStr">
@@ -30257,7 +30257,7 @@
       </c>
       <c r="N370" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O370" t="inlineStr">
@@ -30309,7 +30309,7 @@
       </c>
       <c r="N371" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O371" t="inlineStr">
@@ -30361,7 +30361,7 @@
       </c>
       <c r="N372" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O372" t="inlineStr">
@@ -30413,7 +30413,7 @@
       </c>
       <c r="N373" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O373" t="inlineStr">
@@ -30465,7 +30465,7 @@
       </c>
       <c r="N374" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O374" t="inlineStr">
@@ -30522,7 +30522,7 @@
       </c>
       <c r="N375" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No CASPEX</t>
         </is>
       </c>
       <c r="O375" t="inlineStr">

</xml_diff>

<commit_message>
Edit a guide rule
</commit_message>
<xml_diff>
--- a/cellstocks/data/admin.xlsx
+++ b/cellstocks/data/admin.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -708,7 +708,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -954,7 +954,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -1036,7 +1036,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -1118,7 +1118,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -1282,7 +1282,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -1364,7 +1364,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -1528,7 +1528,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -1610,7 +1610,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -1692,7 +1692,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -1774,7 +1774,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
@@ -1856,7 +1856,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
@@ -1938,7 +1938,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
@@ -2020,7 +2020,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
@@ -2102,7 +2102,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
@@ -2184,7 +2184,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
@@ -2266,7 +2266,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
@@ -2348,7 +2348,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
@@ -2430,7 +2430,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
@@ -2512,7 +2512,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
@@ -2594,7 +2594,7 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
@@ -2676,7 +2676,7 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
@@ -2768,7 +2768,7 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
@@ -2860,7 +2860,7 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
@@ -2952,7 +2952,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
@@ -3044,7 +3044,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
@@ -3126,7 +3126,7 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
@@ -3290,7 +3290,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -3372,7 +3372,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
@@ -3454,7 +3454,7 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -3536,7 +3536,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">
@@ -3700,7 +3700,7 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
@@ -4028,7 +4028,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
@@ -4274,7 +4274,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
@@ -4438,7 +4438,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
@@ -4520,7 +4520,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
@@ -4602,7 +4602,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
@@ -4684,7 +4684,7 @@
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R56" t="inlineStr">
@@ -4766,7 +4766,7 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
@@ -4848,7 +4848,7 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R58" t="inlineStr">
@@ -4930,7 +4930,7 @@
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="P59" t="inlineStr">
@@ -5298,7 +5298,7 @@
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R63" t="inlineStr">
@@ -5380,7 +5380,7 @@
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R64" t="inlineStr">
@@ -5462,7 +5462,7 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R65" t="inlineStr">
@@ -5544,7 +5544,7 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R66" t="inlineStr">
@@ -5626,7 +5626,7 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R67" t="inlineStr">
@@ -5708,7 +5708,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R68" t="inlineStr">
@@ -5790,7 +5790,7 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="P69" t="inlineStr">
@@ -5964,7 +5964,7 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R71" t="inlineStr">
@@ -6128,7 +6128,7 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R73" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R77" t="inlineStr">
@@ -6538,7 +6538,7 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R78" t="inlineStr">
@@ -6620,7 +6620,7 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R79" t="inlineStr">
@@ -6702,7 +6702,7 @@
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R80" t="inlineStr">
@@ -6784,7 +6784,7 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R81" t="inlineStr">
@@ -6866,7 +6866,7 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R82" t="inlineStr">
@@ -6948,7 +6948,7 @@
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R83" t="inlineStr">
@@ -7030,7 +7030,7 @@
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R84" t="inlineStr">
@@ -7112,7 +7112,7 @@
       </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R85" t="inlineStr">
@@ -7194,7 +7194,7 @@
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R86" t="inlineStr">
@@ -7276,7 +7276,7 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R87" t="inlineStr">
@@ -7358,7 +7358,7 @@
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="P88" t="inlineStr">
@@ -7532,7 +7532,7 @@
       </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R90" t="inlineStr">
@@ -7614,7 +7614,7 @@
       </c>
       <c r="O91" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R91" t="inlineStr">
@@ -7696,7 +7696,7 @@
       </c>
       <c r="O92" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R92" t="inlineStr">
@@ -7778,7 +7778,7 @@
       </c>
       <c r="O93" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R93" t="inlineStr">
@@ -7860,7 +7860,7 @@
       </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R94" t="inlineStr">
@@ -8024,7 +8024,7 @@
       </c>
       <c r="O96" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R96" t="inlineStr">
@@ -8106,7 +8106,7 @@
       </c>
       <c r="O97" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R97" t="inlineStr">
@@ -8270,7 +8270,7 @@
       </c>
       <c r="O99" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R99" t="inlineStr">
@@ -8352,7 +8352,7 @@
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R100" t="inlineStr">
@@ -8434,7 +8434,7 @@
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R101" t="inlineStr">
@@ -8516,7 +8516,7 @@
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R102" t="inlineStr">
@@ -8598,7 +8598,7 @@
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R103" t="inlineStr">
@@ -8680,7 +8680,7 @@
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="P104" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R105" t="inlineStr">
@@ -8854,7 +8854,7 @@
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R106" t="inlineStr">
@@ -8936,7 +8936,7 @@
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R107" t="inlineStr">
@@ -9018,7 +9018,7 @@
       </c>
       <c r="O108" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R108" t="inlineStr">
@@ -9100,7 +9100,7 @@
       </c>
       <c r="O109" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R109" t="inlineStr">
@@ -9182,7 +9182,7 @@
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R110" t="inlineStr">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R111" t="inlineStr">
@@ -9346,7 +9346,7 @@
       </c>
       <c r="O112" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R112" t="inlineStr">
@@ -9428,7 +9428,7 @@
       </c>
       <c r="O113" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R113" t="inlineStr">
@@ -9510,7 +9510,7 @@
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R114" t="inlineStr">
@@ -9592,7 +9592,7 @@
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R115" t="inlineStr">
@@ -9674,7 +9674,7 @@
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R116" t="inlineStr">
@@ -9756,7 +9756,7 @@
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R117" t="inlineStr">
@@ -9920,7 +9920,7 @@
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R119" t="inlineStr">
@@ -10002,7 +10002,7 @@
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R120" t="inlineStr">
@@ -10084,7 +10084,7 @@
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R121" t="inlineStr">
@@ -10166,7 +10166,7 @@
       </c>
       <c r="O122" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R122" t="inlineStr">
@@ -10248,7 +10248,7 @@
       </c>
       <c r="O123" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R123" t="inlineStr">
@@ -10494,7 +10494,7 @@
       </c>
       <c r="O126" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R126" t="inlineStr">
@@ -10576,7 +10576,7 @@
       </c>
       <c r="O127" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R127" t="inlineStr">
@@ -10658,7 +10658,7 @@
       </c>
       <c r="O128" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R128" t="inlineStr">
@@ -10740,7 +10740,7 @@
       </c>
       <c r="O129" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R129" t="inlineStr">
@@ -10822,7 +10822,7 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R130" t="inlineStr">
@@ -10904,7 +10904,7 @@
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R131" t="inlineStr">
@@ -10986,7 +10986,7 @@
       </c>
       <c r="O132" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R132" t="inlineStr">
@@ -11068,7 +11068,7 @@
       </c>
       <c r="O133" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R133" t="inlineStr">
@@ -11150,7 +11150,7 @@
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R134" t="inlineStr">
@@ -11232,7 +11232,7 @@
       </c>
       <c r="O135" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R135" t="inlineStr">
@@ -11314,7 +11314,7 @@
       </c>
       <c r="O136" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R136" t="inlineStr">
@@ -11396,7 +11396,7 @@
       </c>
       <c r="O137" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R137" t="inlineStr">
@@ -11478,7 +11478,7 @@
       </c>
       <c r="O138" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R138" t="inlineStr">
@@ -11560,7 +11560,7 @@
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R139" t="inlineStr">
@@ -11970,7 +11970,7 @@
       </c>
       <c r="O144" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R144" t="inlineStr">
@@ -12052,7 +12052,7 @@
       </c>
       <c r="O145" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R145" t="inlineStr">
@@ -12134,7 +12134,7 @@
       </c>
       <c r="O146" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R146" t="inlineStr">
@@ -12216,7 +12216,7 @@
       </c>
       <c r="O147" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R147" t="inlineStr">
@@ -12298,7 +12298,7 @@
       </c>
       <c r="O148" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R148" t="inlineStr">
@@ -12380,7 +12380,7 @@
       </c>
       <c r="O149" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R149" t="inlineStr">
@@ -12969,7 +12969,7 @@
       </c>
       <c r="O156" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R156" t="inlineStr">
@@ -13051,7 +13051,7 @@
       </c>
       <c r="O157" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R157" t="inlineStr">
@@ -13133,7 +13133,7 @@
       </c>
       <c r="O158" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R158" t="inlineStr">
@@ -13215,7 +13215,7 @@
       </c>
       <c r="O159" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R159" t="inlineStr">
@@ -13297,7 +13297,7 @@
       </c>
       <c r="O160" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R160" t="inlineStr">
@@ -13379,7 +13379,7 @@
       </c>
       <c r="O161" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="P161" t="inlineStr">
@@ -13717,7 +13717,7 @@
       </c>
       <c r="O165" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R165" t="inlineStr">
@@ -13799,7 +13799,7 @@
       </c>
       <c r="O166" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R166" t="inlineStr">
@@ -13881,7 +13881,7 @@
       </c>
       <c r="O167" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R167" t="inlineStr">
@@ -14127,7 +14127,7 @@
       </c>
       <c r="O170" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R170" t="inlineStr">
@@ -14209,7 +14209,7 @@
       </c>
       <c r="O171" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R171" t="inlineStr">
@@ -14291,7 +14291,7 @@
       </c>
       <c r="O172" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R172" t="inlineStr">
@@ -14537,7 +14537,7 @@
       </c>
       <c r="O175" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R175" t="inlineStr">
@@ -14619,7 +14619,7 @@
       </c>
       <c r="O176" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R176" t="inlineStr">
@@ -14701,7 +14701,7 @@
       </c>
       <c r="O177" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R177" t="inlineStr">
@@ -14947,7 +14947,7 @@
       </c>
       <c r="O180" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R180" t="inlineStr">
@@ -15029,7 +15029,7 @@
       </c>
       <c r="O181" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="P181" t="inlineStr">
@@ -15121,7 +15121,7 @@
       </c>
       <c r="O182" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R182" t="inlineStr">
@@ -15203,7 +15203,7 @@
       </c>
       <c r="O183" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R183" t="inlineStr">
@@ -15285,7 +15285,7 @@
       </c>
       <c r="O184" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="P184" t="inlineStr">
@@ -15377,7 +15377,7 @@
       </c>
       <c r="O185" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="P185" t="inlineStr">
@@ -15469,7 +15469,7 @@
       </c>
       <c r="O186" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="P186" t="inlineStr">
@@ -15561,7 +15561,7 @@
       </c>
       <c r="O187" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R187" t="inlineStr">
@@ -15643,7 +15643,7 @@
       </c>
       <c r="O188" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R188" t="inlineStr">
@@ -15725,7 +15725,7 @@
       </c>
       <c r="O189" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R189" t="inlineStr">
@@ -15807,7 +15807,7 @@
       </c>
       <c r="O190" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R190" t="inlineStr">
@@ -15889,7 +15889,7 @@
       </c>
       <c r="O191" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R191" t="inlineStr">
@@ -16053,7 +16053,7 @@
       </c>
       <c r="O193" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R193" t="inlineStr">
@@ -16135,7 +16135,7 @@
       </c>
       <c r="O194" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R194" t="inlineStr">
@@ -16217,7 +16217,7 @@
       </c>
       <c r="O195" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R195" t="inlineStr">
@@ -16463,7 +16463,7 @@
       </c>
       <c r="O198" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R198" t="inlineStr">
@@ -16545,7 +16545,7 @@
       </c>
       <c r="O199" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R199" t="inlineStr">
@@ -16627,7 +16627,7 @@
       </c>
       <c r="O200" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R200" t="inlineStr">
@@ -16709,7 +16709,7 @@
       </c>
       <c r="O201" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R201" t="inlineStr">
@@ -16791,7 +16791,7 @@
       </c>
       <c r="O202" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R202" t="inlineStr">
@@ -16873,7 +16873,7 @@
       </c>
       <c r="O203" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R203" t="inlineStr">
@@ -17119,7 +17119,7 @@
       </c>
       <c r="O206" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R206" t="inlineStr">
@@ -17201,7 +17201,7 @@
       </c>
       <c r="O207" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R207" t="inlineStr">
@@ -17283,7 +17283,7 @@
       </c>
       <c r="O208" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R208" t="inlineStr">
@@ -17365,7 +17365,7 @@
       </c>
       <c r="O209" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R209" t="inlineStr">
@@ -17447,7 +17447,7 @@
       </c>
       <c r="O210" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R210" t="inlineStr">
@@ -17529,7 +17529,7 @@
       </c>
       <c r="O211" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="P211" t="inlineStr">
@@ -17621,7 +17621,7 @@
       </c>
       <c r="O212" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R212" t="inlineStr">
@@ -17703,7 +17703,7 @@
       </c>
       <c r="O213" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R213" t="inlineStr">
@@ -19117,7 +19117,7 @@
       </c>
       <c r="O230" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R230" t="inlineStr">
@@ -19281,7 +19281,7 @@
       </c>
       <c r="O232" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R232" t="inlineStr">
@@ -19445,7 +19445,7 @@
       </c>
       <c r="O234" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R234" t="inlineStr">
@@ -19527,7 +19527,7 @@
       </c>
       <c r="O235" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R235" t="inlineStr">
@@ -19691,7 +19691,7 @@
       </c>
       <c r="O237" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R237" t="inlineStr">
@@ -19773,7 +19773,7 @@
       </c>
       <c r="O238" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R238" t="inlineStr">
@@ -19855,7 +19855,7 @@
       </c>
       <c r="O239" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R239" t="inlineStr">
@@ -19932,7 +19932,7 @@
       </c>
       <c r="O240" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R240" t="inlineStr">
@@ -20009,7 +20009,7 @@
       </c>
       <c r="O241" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R241" t="inlineStr">
@@ -20091,7 +20091,7 @@
       </c>
       <c r="O242" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R242" t="inlineStr">
@@ -20173,7 +20173,7 @@
       </c>
       <c r="O243" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R243" t="inlineStr">
@@ -20255,7 +20255,7 @@
       </c>
       <c r="O244" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R244" t="inlineStr">
@@ -20337,7 +20337,7 @@
       </c>
       <c r="O245" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R245" t="inlineStr">
@@ -20414,7 +20414,7 @@
       </c>
       <c r="O246" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R246" t="inlineStr">
@@ -20578,7 +20578,7 @@
       </c>
       <c r="O248" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R248" t="inlineStr">
@@ -20660,7 +20660,7 @@
       </c>
       <c r="O249" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R249" t="inlineStr">
@@ -20742,7 +20742,7 @@
       </c>
       <c r="O250" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R250" t="inlineStr">
@@ -20824,7 +20824,7 @@
       </c>
       <c r="O251" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R251" t="inlineStr">
@@ -20906,7 +20906,7 @@
       </c>
       <c r="O252" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R252" t="inlineStr">
@@ -21070,7 +21070,7 @@
       </c>
       <c r="O254" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R254" t="inlineStr">
@@ -21152,7 +21152,7 @@
       </c>
       <c r="O255" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R255" t="inlineStr">
@@ -21316,7 +21316,7 @@
       </c>
       <c r="O257" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R257" t="inlineStr">
@@ -21398,7 +21398,7 @@
       </c>
       <c r="O258" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R258" t="inlineStr">
@@ -21480,7 +21480,7 @@
       </c>
       <c r="O259" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R259" t="inlineStr">
@@ -21562,7 +21562,7 @@
       </c>
       <c r="O260" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R260" t="inlineStr">
@@ -22290,7 +22290,7 @@
       </c>
       <c r="O269" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R269" t="inlineStr">
@@ -22372,7 +22372,7 @@
       </c>
       <c r="O270" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R270" t="inlineStr">
@@ -22454,7 +22454,7 @@
       </c>
       <c r="O271" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R271" t="inlineStr">
@@ -22536,7 +22536,7 @@
       </c>
       <c r="O272" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R272" t="inlineStr">
@@ -22618,7 +22618,7 @@
       </c>
       <c r="O273" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R273" t="inlineStr">
@@ -22700,7 +22700,7 @@
       </c>
       <c r="O274" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R274" t="inlineStr">
@@ -22782,7 +22782,7 @@
       </c>
       <c r="O275" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R275" t="inlineStr">
@@ -24335,7 +24335,7 @@
       </c>
       <c r="O294" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R294" t="inlineStr">
@@ -24417,7 +24417,7 @@
       </c>
       <c r="O295" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R295" t="inlineStr">
@@ -24909,7 +24909,7 @@
       </c>
       <c r="O301" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R301" t="inlineStr">
@@ -25319,7 +25319,7 @@
       </c>
       <c r="O306" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R306" t="inlineStr">
@@ -25401,7 +25401,7 @@
       </c>
       <c r="O307" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R307" t="inlineStr">
@@ -25811,7 +25811,7 @@
       </c>
       <c r="O312" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R312" t="inlineStr">
@@ -25975,7 +25975,7 @@
       </c>
       <c r="O314" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R314" t="inlineStr">
@@ -26139,7 +26139,7 @@
       </c>
       <c r="O316" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R316" t="inlineStr">
@@ -26221,7 +26221,7 @@
       </c>
       <c r="O317" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R317" t="inlineStr">
@@ -26385,7 +26385,7 @@
       </c>
       <c r="O319" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R319" t="inlineStr">
@@ -26467,7 +26467,7 @@
       </c>
       <c r="O320" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R320" t="inlineStr">
@@ -27205,7 +27205,7 @@
       </c>
       <c r="O329" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R329" t="inlineStr">
@@ -27635,7 +27635,7 @@
       </c>
       <c r="O334" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R334" t="inlineStr">
@@ -27717,7 +27717,7 @@
       </c>
       <c r="O335" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R335" t="inlineStr">
@@ -27799,7 +27799,7 @@
       </c>
       <c r="O336" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R336" t="inlineStr">
@@ -27876,7 +27876,7 @@
       </c>
       <c r="O337" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R337" t="inlineStr">
@@ -27958,7 +27958,7 @@
       </c>
       <c r="O338" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R338" t="inlineStr">
@@ -28286,7 +28286,7 @@
       </c>
       <c r="O342" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R342" t="inlineStr">
@@ -28368,7 +28368,7 @@
       </c>
       <c r="O343" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R343" t="inlineStr">
@@ -28614,7 +28614,7 @@
       </c>
       <c r="O346" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R346" t="inlineStr">
@@ -28696,7 +28696,7 @@
       </c>
       <c r="O347" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R347" t="inlineStr">
@@ -29270,7 +29270,7 @@
       </c>
       <c r="O354" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R354" t="inlineStr">
@@ -29352,7 +29352,7 @@
       </c>
       <c r="O355" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R355" t="inlineStr">
@@ -29496,7 +29496,7 @@
       </c>
       <c r="O357" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R357" t="inlineStr">
@@ -29620,7 +29620,7 @@
       </c>
       <c r="O359" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R359" t="inlineStr">
@@ -29682,7 +29682,7 @@
       </c>
       <c r="O360" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R360" t="inlineStr">
@@ -29744,7 +29744,7 @@
       </c>
       <c r="O361" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R361" t="inlineStr">
@@ -29868,7 +29868,7 @@
       </c>
       <c r="O363" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R363" t="inlineStr">
@@ -29930,7 +29930,7 @@
       </c>
       <c r="O364" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R364" t="inlineStr">
@@ -29992,7 +29992,7 @@
       </c>
       <c r="O365" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R365" t="inlineStr">
@@ -30054,7 +30054,7 @@
       </c>
       <c r="O366" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R366" t="inlineStr">
@@ -30106,7 +30106,7 @@
       </c>
       <c r="O367" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R367" t="inlineStr">
@@ -30158,7 +30158,7 @@
       </c>
       <c r="O368" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R368" t="inlineStr">
@@ -30210,7 +30210,7 @@
       </c>
       <c r="O369" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R369" t="inlineStr">
@@ -30262,7 +30262,7 @@
       </c>
       <c r="O370" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R370" t="inlineStr">
@@ -30314,7 +30314,7 @@
       </c>
       <c r="O371" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R371" t="inlineStr">
@@ -30366,7 +30366,7 @@
       </c>
       <c r="O372" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R372" t="inlineStr">
@@ -30418,7 +30418,7 @@
       </c>
       <c r="O373" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R373" t="inlineStr">
@@ -30470,7 +30470,7 @@
       </c>
       <c r="O374" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R374" t="inlineStr">
@@ -30527,7 +30527,7 @@
       </c>
       <c r="O375" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R375" t="inlineStr">

</xml_diff>

<commit_message>
Import 157 vials from primers.xlsx from unknown device
</commit_message>
<xml_diff>
--- a/cellstocks/data/admin.xlsx
+++ b/cellstocks/data/admin.xlsx
@@ -37585,6 +37585,228 @@
         <v>81</v>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not placed yet</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not placed yet</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ChIP Box</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">grid</t>
+        </is>
+      </c>
+      <c r="F19">
+        <v>9</v>
+      </c>
+      <c r="G19">
+        <v>9</v>
+      </c>
+      <c r="H19">
+        <v>81</v>
+      </c>
+      <c r="I19">
+        <v>0</v>
+      </c>
+      <c r="J19">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not placed yet</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not placed yet</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ChIP Box -2-</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">grid</t>
+        </is>
+      </c>
+      <c r="F20">
+        <v>9</v>
+      </c>
+      <c r="G20">
+        <v>9</v>
+      </c>
+      <c r="H20">
+        <v>81</v>
+      </c>
+      <c r="I20">
+        <v>0</v>
+      </c>
+      <c r="J20">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not placed yet</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not placed yet</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Umut -20 -2-</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">grid</t>
+        </is>
+      </c>
+      <c r="F21">
+        <v>9</v>
+      </c>
+      <c r="G21">
+        <v>9</v>
+      </c>
+      <c r="H21">
+        <v>81</v>
+      </c>
+      <c r="I21">
+        <v>0</v>
+      </c>
+      <c r="J21">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not placed yet</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not placed yet</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Umut -20 Box -1-</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">grid</t>
+        </is>
+      </c>
+      <c r="F22">
+        <v>9</v>
+      </c>
+      <c r="G22">
+        <v>9</v>
+      </c>
+      <c r="H22">
+        <v>81</v>
+      </c>
+      <c r="I22">
+        <v>0</v>
+      </c>
+      <c r="J22">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not placed yet</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not placed yet</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unkown FOR NOW</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">grid</t>
+        </is>
+      </c>
+      <c r="F23">
+        <v>9</v>
+      </c>
+      <c r="G23">
+        <v>9</v>
+      </c>
+      <c r="H23">
+        <v>81</v>
+      </c>
+      <c r="I23">
+        <v>0</v>
+      </c>
+      <c r="J23">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not placed yet</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not placed yet</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No use</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">grid</t>
+        </is>
+      </c>
+      <c r="F24">
+        <v>9</v>
+      </c>
+      <c r="G24">
+        <v>9</v>
+      </c>
+      <c r="H24">
+        <v>81</v>
+      </c>
+      <c r="I24">
+        <v>0</v>
+      </c>
+      <c r="J24">
+        <v>81</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Move ChIP Box -2-
</commit_message>
<xml_diff>
--- a/cellstocks/data/admin.xlsx
+++ b/cellstocks/data/admin.xlsx
@@ -39361,17 +39361,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 2</t>
+          <t xml:space="preserve">Fridge 1</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Baris Shelf</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">-80 Box1</t>
+          <t xml:space="preserve">ChIP Box -2-</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -39408,7 +39408,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">-80 Box2</t>
+          <t xml:space="preserve">-80 Box1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -39445,7 +39445,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">-80 Box3</t>
+          <t xml:space="preserve">-80 Box2</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -39482,7 +39482,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">-80 Box4</t>
+          <t xml:space="preserve">-80 Box3</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -39519,7 +39519,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">-80 Box5</t>
+          <t xml:space="preserve">-80 Box4</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -39556,7 +39556,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">-80 Box6</t>
+          <t xml:space="preserve">-80 Box5</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -39588,12 +39588,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Beyza Shelf</t>
+          <t xml:space="preserve">Baris Shelf</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Beyza Caa Hücre Box 2</t>
+          <t xml:space="preserve">-80 Box6</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -39620,17 +39620,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Freezer 2</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Beyza Shelf</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">ChIP Box -2-</t>
+          <t xml:space="preserve">Beyza Caa Hücre Box 2</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">

</xml_diff>

<commit_message>
Move Umut -20 -2-
</commit_message>
<xml_diff>
--- a/cellstocks/data/admin.xlsx
+++ b/cellstocks/data/admin.xlsx
@@ -39398,17 +39398,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 2</t>
+          <t xml:space="preserve">Fridge 1</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Baris Shelf</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">-80 Box1</t>
+          <t xml:space="preserve">Umut -20 -2-</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -39445,7 +39445,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">-80 Box2</t>
+          <t xml:space="preserve">-80 Box1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -39482,7 +39482,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">-80 Box3</t>
+          <t xml:space="preserve">-80 Box2</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -39519,7 +39519,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">-80 Box4</t>
+          <t xml:space="preserve">-80 Box3</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -39556,7 +39556,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">-80 Box5</t>
+          <t xml:space="preserve">-80 Box4</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -39593,7 +39593,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">-80 Box6</t>
+          <t xml:space="preserve">-80 Box5</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -39625,12 +39625,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Beyza Shelf</t>
+          <t xml:space="preserve">Baris Shelf</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Beyza Caa Hücre Box 2</t>
+          <t xml:space="preserve">-80 Box6</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -39657,17 +39657,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Freezer 2</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Beyza Shelf</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Umut -20 -2-</t>
+          <t xml:space="preserve">Beyza Caa Hücre Box 2</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">

</xml_diff>

<commit_message>
Move Umut -20 Box -1-
</commit_message>
<xml_diff>
--- a/cellstocks/data/admin.xlsx
+++ b/cellstocks/data/admin.xlsx
@@ -39435,17 +39435,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Freezer 2</t>
+          <t xml:space="preserve">Fridge 1</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Baris Shelf</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">-80 Box1</t>
+          <t xml:space="preserve">Umut -20 Box -1-</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -39482,7 +39482,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">-80 Box2</t>
+          <t xml:space="preserve">-80 Box1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -39519,7 +39519,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">-80 Box3</t>
+          <t xml:space="preserve">-80 Box2</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -39556,7 +39556,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">-80 Box4</t>
+          <t xml:space="preserve">-80 Box3</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -39593,7 +39593,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">-80 Box5</t>
+          <t xml:space="preserve">-80 Box4</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -39630,7 +39630,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">-80 Box6</t>
+          <t xml:space="preserve">-80 Box5</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -39662,12 +39662,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Beyza Shelf</t>
+          <t xml:space="preserve">Baris Shelf</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Beyza Caa Hücre Box 2</t>
+          <t xml:space="preserve">-80 Box6</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -39694,17 +39694,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Freezer 2</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Beyza Shelf</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Umut -20 Box -1-</t>
+          <t xml:space="preserve">Beyza Caa Hücre Box 2</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">

</xml_diff>

<commit_message>
Admin: added a box for Umut
</commit_message>
<xml_diff>
--- a/cellstocks/data/admin.xlsx
+++ b/cellstocks/data/admin.xlsx
@@ -37556,12 +37556,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -37588,17 +37588,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fridge 1</t>
+          <t xml:space="preserve">Freezer 1</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 1</t>
+          <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">ChIP Box</t>
+          <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -37635,7 +37635,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">ChIP Box -2-</t>
+          <t xml:space="preserve">ChIP Box</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -37672,7 +37672,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Umut -20 -2-</t>
+          <t xml:space="preserve">ChIP Box -2-</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -37709,7 +37709,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Umut -20 Box -1-</t>
+          <t xml:space="preserve">Umut -20 -2-</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -37736,17 +37736,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Fridge 1</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unkown FOR NOW</t>
+          <t xml:space="preserve">Umut -20 Box -1-</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -37783,7 +37783,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve">No use</t>
+          <t xml:space="preserve">Unkown FOR NOW</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -37804,6 +37804,43 @@
         <v>0</v>
       </c>
       <c r="J24">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not placed yet</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not placed yet</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No use</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">grid</t>
+        </is>
+      </c>
+      <c r="F25">
+        <v>9</v>
+      </c>
+      <c r="G25">
+        <v>9</v>
+      </c>
+      <c r="H25">
+        <v>81</v>
+      </c>
+      <c r="I25">
+        <v>0</v>
+      </c>
+      <c r="J25">
         <v>81</v>
       </c>
     </row>

</xml_diff>